<commit_message>
Euro NCAP Rating Calculator 2026, version 5.4.9
</commit_message>
<xml_diff>
--- a/data/cp_template.xlsx
+++ b/data/cp_template.xlsx
@@ -1604,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25.63" customWidth="1" style="126" min="1" max="1"/>
@@ -1724,7 +1724,7 @@
       <c r="C8" s="139" t="n"/>
       <c r="D8" s="127" t="inlineStr">
         <is>
-          <t>Red line &gt;125 mm outboard of the orange line</t>
+          <t>Red line &gt;125 mm outboard of the orange line ?</t>
         </is>
       </c>
       <c r="E8" s="142" t="n"/>
@@ -1743,58 +1743,69 @@
       </c>
       <c r="D9" s="127" t="inlineStr">
         <is>
-          <t>Torso angle (rear)</t>
+          <t>Torso angle (rear second row)</t>
         </is>
       </c>
       <c r="E9" s="142" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="129">
       <c r="A10" s="138" t="n"/>
-      <c r="B10" s="141" t="inlineStr">
+      <c r="B10" s="141" t="n"/>
+      <c r="C10" s="139" t="n"/>
+      <c r="D10" s="127" t="inlineStr">
+        <is>
+          <t>Torso angle (rear third row)</t>
+        </is>
+      </c>
+      <c r="E10" s="142" t="n"/>
+    </row>
+    <row r="11" ht="14.25" customHeight="1" s="129">
+      <c r="A11" s="138" t="n"/>
+      <c r="B11" s="141" t="inlineStr">
         <is>
           <t>VRU Impact</t>
         </is>
       </c>
-      <c r="C10" s="139" t="inlineStr">
+      <c r="C11" s="139" t="inlineStr">
         <is>
           <t>Head Impact</t>
         </is>
       </c>
-      <c r="D10" s="127" t="inlineStr">
+      <c r="D11" s="127" t="inlineStr">
         <is>
           <t>Number of verification tests (min 10)</t>
         </is>
       </c>
-      <c r="E10" s="143" t="n"/>
-    </row>
-    <row r="11" ht="14.25" customHeight="1" s="129">
-      <c r="A11" s="127" t="n"/>
-      <c r="C11" s="139" t="inlineStr">
+      <c r="E11" s="143" t="n"/>
+    </row>
+    <row r="12" ht="14.25" customHeight="1" s="129">
+      <c r="A12" s="127" t="n"/>
+      <c r="C12" s="139" t="inlineStr">
         <is>
           <t>Pelvis Impact</t>
         </is>
       </c>
-      <c r="D11" s="127" t="inlineStr">
+      <c r="D12" s="127" t="inlineStr">
         <is>
           <t>Number of verification tests (min 5)</t>
         </is>
       </c>
-      <c r="E11" s="143" t="n"/>
-    </row>
-    <row r="12" ht="14.25" customHeight="1" s="129">
-      <c r="A12" s="144" t="n"/>
-      <c r="B12" s="145" t="n"/>
-      <c r="C12" s="146" t="inlineStr">
+      <c r="E12" s="143" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="144" t="n"/>
+      <c r="B13" s="145" t="n"/>
+      <c r="C13" s="146" t="inlineStr">
         <is>
           <t>Leg Impact</t>
         </is>
       </c>
-      <c r="D12" s="145" t="inlineStr">
+      <c r="D13" s="145" t="inlineStr">
         <is>
           <t>Number of verification tests (min 5)</t>
         </is>
       </c>
-      <c r="E12" s="147" t="n"/>
+      <c r="E13" s="147" t="n"/>
     </row>
     <row r="1048557" ht="12.75" customHeight="1" s="129"/>
     <row r="1048558" ht="12.75" customHeight="1" s="129"/>
@@ -2786,7 +2797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.64" customWidth="1" style="126" min="1" max="2"/>
@@ -3499,7 +3510,7 @@
       </c>
       <c r="B39" s="172" t="inlineStr">
         <is>
-          <t>Rear</t>
+          <t>Rear (second row)</t>
         </is>
       </c>
       <c r="C39" s="172" t="inlineStr">
@@ -3547,7 +3558,7 @@
       <c r="A41" s="153" t="n"/>
       <c r="E41" s="126" t="inlineStr">
         <is>
-          <t>Effective height modifier</t>
+          <t>Non-Use position</t>
         </is>
       </c>
       <c r="I41" s="202" t="n"/>
@@ -3586,6 +3597,95 @@
       </c>
       <c r="H43" s="197" t="n"/>
       <c r="I43" s="207" t="n"/>
+    </row>
+    <row r="44" ht="14.25" customHeight="1" s="129">
+      <c r="A44" s="210" t="n"/>
+      <c r="B44" s="172" t="inlineStr">
+        <is>
+          <t>Rear (third row)</t>
+        </is>
+      </c>
+      <c r="C44" s="172" t="inlineStr">
+        <is>
+          <t>HPM</t>
+        </is>
+      </c>
+      <c r="D44" s="172" t="inlineStr">
+        <is>
+          <t>Neck</t>
+        </is>
+      </c>
+      <c r="E44" s="172" t="inlineStr">
+        <is>
+          <t>Effective height - Lowest</t>
+        </is>
+      </c>
+      <c r="F44" s="211" t="n">
+        <v>720</v>
+      </c>
+      <c r="G44" s="211" t="n">
+        <v>719.99</v>
+      </c>
+      <c r="H44" s="211" t="n"/>
+      <c r="I44" s="202" t="n"/>
+    </row>
+    <row r="45" ht="14.25" customHeight="1" s="129">
+      <c r="A45" s="153" t="n"/>
+      <c r="E45" s="126" t="inlineStr">
+        <is>
+          <t>Effective height - Highest</t>
+        </is>
+      </c>
+      <c r="F45" s="128" t="n">
+        <v>770</v>
+      </c>
+      <c r="G45" s="128" t="n">
+        <v>769.99</v>
+      </c>
+      <c r="I45" s="202" t="n"/>
+    </row>
+    <row r="46" ht="14.25" customHeight="1" s="129">
+      <c r="A46" s="153" t="n"/>
+      <c r="E46" s="126" t="inlineStr">
+        <is>
+          <t>Non-Use position</t>
+        </is>
+      </c>
+      <c r="I46" s="202" t="n"/>
+    </row>
+    <row r="47" ht="14.25" customHeight="1" s="129">
+      <c r="A47" s="153" t="n"/>
+      <c r="E47" s="126" t="inlineStr">
+        <is>
+          <t>Backset - Lowest</t>
+        </is>
+      </c>
+      <c r="F47" s="128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="202" t="n"/>
+    </row>
+    <row r="48" ht="14.25" customHeight="1" s="129">
+      <c r="A48" s="164" t="n"/>
+      <c r="B48" s="165" t="n"/>
+      <c r="C48" s="165" t="n"/>
+      <c r="D48" s="165" t="n"/>
+      <c r="E48" s="165" t="inlineStr">
+        <is>
+          <t>Backset - Mid</t>
+        </is>
+      </c>
+      <c r="F48" s="197" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="197" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="197" t="n"/>
+      <c r="I48" s="207" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -5033,7 +5133,7 @@
       </c>
       <c r="B1" s="256" t="inlineStr">
         <is>
-          <t>5.4.7</t>
+          <t>5.4.9</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18.63" customWidth="1" style="126" min="1" max="1"/>
@@ -6250,7 +6350,7 @@
       </c>
       <c r="E30" s="126" t="inlineStr">
         <is>
-          <t>Front</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="F30" s="126" t="inlineStr">
@@ -6269,175 +6369,231 @@
         </is>
       </c>
       <c r="I30" s="157" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="31" ht="14.25" customHeight="1" s="129">
-      <c r="A31" s="164" t="n"/>
-      <c r="B31" s="165" t="n"/>
-      <c r="C31" s="165" t="n"/>
-      <c r="D31" s="165" t="inlineStr">
+      <c r="A31" s="153" t="n"/>
+      <c r="D31" s="126" t="n"/>
+      <c r="E31" s="126" t="inlineStr">
+        <is>
+          <t>Front Passenger</t>
+        </is>
+      </c>
+      <c r="F31" s="126" t="inlineStr">
+        <is>
+          <t>HPM</t>
+        </is>
+      </c>
+      <c r="G31" s="155" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H31" s="156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I31" s="157" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="32" ht="14.25" customHeight="1" s="129">
+      <c r="A32" s="164" t="n"/>
+      <c r="B32" s="165" t="n"/>
+      <c r="C32" s="165" t="n"/>
+      <c r="D32" s="165" t="inlineStr">
         <is>
           <t>Static-Rear</t>
         </is>
       </c>
-      <c r="E31" s="165" t="inlineStr">
-        <is>
-          <t>Rear</t>
-        </is>
-      </c>
-      <c r="F31" s="165" t="inlineStr">
+      <c r="E32" s="165" t="inlineStr">
+        <is>
+          <t>Rear (second row)</t>
+        </is>
+      </c>
+      <c r="F32" s="165" t="inlineStr">
         <is>
           <t>HPM</t>
         </is>
       </c>
-      <c r="G31" s="166" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H31" s="167" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I31" s="168" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" ht="14.25" customHeight="1" s="129">
-      <c r="A32" s="169" t="inlineStr">
+      <c r="G32" s="166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" s="167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" s="168" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="33" ht="14.25" customHeight="1" s="129">
+      <c r="A33" s="164" t="n"/>
+      <c r="B33" s="165" t="n"/>
+      <c r="C33" s="165" t="n"/>
+      <c r="D33" s="165" t="n"/>
+      <c r="E33" s="165" t="inlineStr">
+        <is>
+          <t>Rear (third row)</t>
+        </is>
+      </c>
+      <c r="F33" s="165" t="inlineStr">
+        <is>
+          <t>HPM</t>
+        </is>
+      </c>
+      <c r="G33" s="166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H33" s="167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I33" s="168" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="34" ht="14.25" customHeight="1" s="129">
+      <c r="A34" s="169" t="inlineStr">
         <is>
           <t>Crash Protection</t>
         </is>
       </c>
-      <c r="B32" s="176" t="inlineStr">
+      <c r="B34" s="176" t="inlineStr">
         <is>
           <t>VRU Impact</t>
         </is>
       </c>
-      <c r="C32" s="176" t="inlineStr">
+      <c r="C34" s="176" t="inlineStr">
         <is>
           <t>Head Impact</t>
         </is>
       </c>
-      <c r="D32" s="176" t="inlineStr">
+      <c r="D34" s="176" t="inlineStr">
         <is>
           <t>Headform</t>
         </is>
       </c>
-      <c r="E32" s="176" t="inlineStr">
+      <c r="E34" s="176" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="F32" s="176" t="inlineStr">
+      <c r="F34" s="176" t="inlineStr">
         <is>
           <t>Adult Headform</t>
         </is>
       </c>
-      <c r="G32" s="176" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H32" s="180" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I32" s="179" t="n"/>
-    </row>
-    <row r="33" ht="14.25" customHeight="1" s="129">
-      <c r="A33" s="153" t="n"/>
-      <c r="E33" s="126" t="inlineStr">
+      <c r="G34" s="176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" s="179" t="n"/>
+    </row>
+    <row r="35" ht="14.25" customHeight="1" s="129">
+      <c r="A35" s="153" t="n"/>
+      <c r="E35" s="126" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="F33" s="126" t="inlineStr">
+      <c r="F35" s="126" t="inlineStr">
         <is>
           <t>Child Headform</t>
         </is>
       </c>
-      <c r="G33" s="126" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H33" s="181" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I33" s="157" t="n"/>
-    </row>
-    <row r="34" ht="14.25" customHeight="1" s="129">
-      <c r="A34" s="153" t="n"/>
-      <c r="C34" s="172" t="inlineStr">
+      <c r="G35" s="126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="157" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="153" t="n"/>
+      <c r="C36" s="172" t="inlineStr">
         <is>
           <t>Pelvis &amp; Leg Impact</t>
         </is>
       </c>
-      <c r="D34" s="172" t="inlineStr">
+      <c r="D36" s="172" t="inlineStr">
         <is>
           <t>Upper Leg</t>
         </is>
       </c>
-      <c r="E34" s="172" t="inlineStr">
+      <c r="E36" s="172" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="F34" s="172" t="inlineStr">
+      <c r="F36" s="172" t="inlineStr">
         <is>
           <t>Upper legform</t>
         </is>
       </c>
-      <c r="G34" s="172" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H34" s="182" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I34" s="175" t="n">
+      <c r="G36" s="172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="182" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I36" s="175" t="n">
         <v>2.5</v>
       </c>
     </row>
-    <row r="35" ht="14.25" customHeight="1" s="129">
-      <c r="A35" s="164" t="n"/>
-      <c r="B35" s="165" t="n"/>
-      <c r="C35" s="165" t="n"/>
-      <c r="D35" s="165" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="164" t="n"/>
+      <c r="B37" s="165" t="n"/>
+      <c r="C37" s="165" t="n"/>
+      <c r="D37" s="165" t="inlineStr">
         <is>
           <t>Lower Leg</t>
         </is>
       </c>
-      <c r="E35" s="165" t="inlineStr">
+      <c r="E37" s="165" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="F35" s="165" t="inlineStr">
+      <c r="F37" s="165" t="inlineStr">
         <is>
           <t>aPLI</t>
         </is>
       </c>
-      <c r="G35" s="165" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H35" s="183" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I35" s="168" t="n">
+      <c r="G37" s="165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H37" s="183" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I37" s="168" t="n">
         <v>7.5</v>
       </c>
     </row>
@@ -6463,7 +6619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S98"/>
+  <dimension ref="A1:S100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.64" customWidth="1" style="126" min="1" max="1"/>
@@ -9330,7 +9486,7 @@
       </c>
       <c r="D88" s="126" t="inlineStr">
         <is>
-          <t>Front</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="E88" s="126" t="inlineStr">
@@ -9360,157 +9516,172 @@
         </is>
       </c>
       <c r="K88" s="157" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1" s="129">
-      <c r="A89" s="164" t="n"/>
-      <c r="B89" s="165" t="n"/>
-      <c r="C89" s="165" t="inlineStr">
+      <c r="A89" s="153" t="n"/>
+      <c r="C89" s="126" t="n"/>
+      <c r="D89" s="126" t="inlineStr">
+        <is>
+          <t>Front Passenger</t>
+        </is>
+      </c>
+      <c r="E89" s="126" t="inlineStr">
+        <is>
+          <t>HPM</t>
+        </is>
+      </c>
+      <c r="F89" s="126" t="inlineStr">
+        <is>
+          <t>Neck</t>
+        </is>
+      </c>
+      <c r="G89" s="187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H89" s="187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I89" s="187" t="n"/>
+      <c r="J89" s="156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K89" s="157" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="90" ht="14.25" customHeight="1" s="129">
+      <c r="A90" s="164" t="n"/>
+      <c r="B90" s="165" t="n"/>
+      <c r="C90" s="165" t="inlineStr">
         <is>
           <t>Static-Rear</t>
         </is>
       </c>
-      <c r="D89" s="165" t="inlineStr">
-        <is>
-          <t>Rear</t>
-        </is>
-      </c>
-      <c r="E89" s="165" t="inlineStr">
+      <c r="D90" s="165" t="inlineStr">
+        <is>
+          <t>Rear (second row)</t>
+        </is>
+      </c>
+      <c r="E90" s="165" t="inlineStr">
         <is>
           <t>HPM</t>
         </is>
       </c>
-      <c r="F89" s="165" t="inlineStr">
+      <c r="F90" s="165" t="inlineStr">
         <is>
           <t>Neck</t>
         </is>
       </c>
-      <c r="G89" s="188" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H89" s="188" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I89" s="188" t="n"/>
-      <c r="J89" s="167" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K89" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="M89" s="191" t="n"/>
-      <c r="N89" s="191" t="n"/>
-      <c r="O89" s="191" t="n"/>
-      <c r="P89" s="191" t="n"/>
-      <c r="Q89" s="191" t="n"/>
-      <c r="R89" s="191" t="n"/>
-      <c r="S89" s="191" t="n"/>
-    </row>
-    <row r="90" ht="14.25" customHeight="1" s="129">
-      <c r="A90" s="126" t="inlineStr">
+      <c r="G90" s="188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H90" s="188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I90" s="188" t="n"/>
+      <c r="J90" s="167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K90" s="168" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M90" s="191" t="n"/>
+      <c r="N90" s="191" t="n"/>
+      <c r="O90" s="191" t="n"/>
+      <c r="P90" s="191" t="n"/>
+      <c r="Q90" s="191" t="n"/>
+      <c r="R90" s="191" t="n"/>
+      <c r="S90" s="191" t="n"/>
+    </row>
+    <row r="91" ht="14.25" customHeight="1" s="129">
+      <c r="A91" s="164" t="n"/>
+      <c r="B91" s="165" t="n"/>
+      <c r="C91" s="165" t="n"/>
+      <c r="D91" s="165" t="inlineStr">
+        <is>
+          <t>Rear (third row)</t>
+        </is>
+      </c>
+      <c r="E91" s="165" t="inlineStr">
+        <is>
+          <t>HPM</t>
+        </is>
+      </c>
+      <c r="F91" s="165" t="inlineStr">
+        <is>
+          <t>Neck</t>
+        </is>
+      </c>
+      <c r="G91" s="188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H91" s="188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I91" s="188" t="n"/>
+      <c r="J91" s="167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K91" s="168" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M91" s="191" t="n"/>
+      <c r="N91" s="191" t="n"/>
+      <c r="O91" s="191" t="n"/>
+      <c r="P91" s="191" t="n"/>
+      <c r="Q91" s="191" t="n"/>
+      <c r="R91" s="191" t="n"/>
+      <c r="S91" s="191" t="n"/>
+    </row>
+    <row r="92" ht="14.25" customHeight="1" s="129">
+      <c r="A92" s="126" t="inlineStr">
         <is>
           <t>VRU Impact</t>
         </is>
       </c>
-      <c r="B90" s="126" t="inlineStr">
+      <c r="B92" s="126" t="inlineStr">
         <is>
           <t>Head Impact</t>
         </is>
       </c>
-      <c r="C90" s="126" t="inlineStr">
+      <c r="C92" s="126" t="inlineStr">
         <is>
           <t>Headform</t>
         </is>
       </c>
-      <c r="D90" s="126" t="inlineStr">
+      <c r="D92" s="126" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="E90" s="126" t="inlineStr">
+      <c r="E92" s="126" t="inlineStr">
         <is>
           <t>Adult Headform</t>
         </is>
       </c>
-      <c r="F90" s="126" t="inlineStr">
+      <c r="F92" s="126" t="inlineStr">
         <is>
           <t>Cyclist</t>
-        </is>
-      </c>
-      <c r="G90" s="192" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H90" s="126" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J90" s="156" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K90" s="157" t="n"/>
-      <c r="M90" s="193" t="n"/>
-      <c r="N90" s="193" t="n"/>
-      <c r="O90" s="193" t="n"/>
-      <c r="P90" s="193" t="n"/>
-      <c r="Q90" s="193" t="n"/>
-      <c r="R90" s="193" t="n"/>
-      <c r="S90" s="193" t="n"/>
-    </row>
-    <row r="91" ht="14.25" customHeight="1" s="129">
-      <c r="A91" s="126" t="n"/>
-      <c r="F91" s="126" t="inlineStr">
-        <is>
-          <t>Adult</t>
-        </is>
-      </c>
-      <c r="G91" s="192" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H91" s="126" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J91" s="156" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K91" s="157" t="n"/>
-      <c r="M91" s="193" t="n"/>
-      <c r="N91" s="193" t="n"/>
-      <c r="O91" s="193" t="n"/>
-      <c r="P91" s="193" t="n"/>
-    </row>
-    <row r="92" ht="14.25" customHeight="1" s="129">
-      <c r="A92" s="126" t="n"/>
-      <c r="D92" s="126" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="E92" s="126" t="inlineStr">
-        <is>
-          <t>Child Headform</t>
-        </is>
-      </c>
-      <c r="F92" s="126" t="inlineStr">
-        <is>
-          <t>Child</t>
         </is>
       </c>
       <c r="G92" s="192" t="inlineStr">
@@ -9533,137 +9704,207 @@
       <c r="N92" s="193" t="n"/>
       <c r="O92" s="193" t="n"/>
       <c r="P92" s="193" t="n"/>
+      <c r="Q92" s="193" t="n"/>
+      <c r="R92" s="193" t="n"/>
+      <c r="S92" s="193" t="n"/>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="129">
       <c r="A93" s="126" t="n"/>
-      <c r="B93" s="176" t="inlineStr">
-        <is>
-          <t>Pelvis &amp; Leg Impact</t>
-        </is>
-      </c>
-      <c r="C93" s="176" t="inlineStr">
-        <is>
-          <t>Upper Leg</t>
-        </is>
-      </c>
-      <c r="D93" s="176" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="E93" s="176" t="inlineStr">
-        <is>
-          <t>Upper legform</t>
-        </is>
-      </c>
-      <c r="F93" s="176" t="inlineStr">
-        <is>
-          <t>Pelvis</t>
-        </is>
-      </c>
-      <c r="G93" s="194" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H93" s="195" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I93" s="195" t="n"/>
-      <c r="J93" s="178" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K93" s="179" t="n">
-        <v>2.5</v>
-      </c>
+      <c r="F93" s="126" t="inlineStr">
+        <is>
+          <t>Adult</t>
+        </is>
+      </c>
+      <c r="G93" s="192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H93" s="126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J93" s="156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K93" s="157" t="n"/>
+      <c r="M93" s="193" t="n"/>
+      <c r="N93" s="193" t="n"/>
+      <c r="O93" s="193" t="n"/>
+      <c r="P93" s="193" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1" s="129">
       <c r="A94" s="126" t="n"/>
-      <c r="C94" s="126" t="inlineStr">
+      <c r="D94" s="126" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="E94" s="126" t="inlineStr">
+        <is>
+          <t>Child Headform</t>
+        </is>
+      </c>
+      <c r="F94" s="126" t="inlineStr">
+        <is>
+          <t>Child</t>
+        </is>
+      </c>
+      <c r="G94" s="192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H94" s="126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J94" s="156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K94" s="157" t="n"/>
+      <c r="M94" s="193" t="n"/>
+      <c r="N94" s="193" t="n"/>
+      <c r="O94" s="193" t="n"/>
+      <c r="P94" s="193" t="n"/>
+    </row>
+    <row r="95" ht="14.25" customHeight="1" s="129">
+      <c r="A95" s="126" t="n"/>
+      <c r="B95" s="176" t="inlineStr">
+        <is>
+          <t>Pelvis &amp; Leg Impact</t>
+        </is>
+      </c>
+      <c r="C95" s="176" t="inlineStr">
+        <is>
+          <t>Upper Leg</t>
+        </is>
+      </c>
+      <c r="D95" s="176" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="E95" s="176" t="inlineStr">
+        <is>
+          <t>Upper legform</t>
+        </is>
+      </c>
+      <c r="F95" s="176" t="inlineStr">
+        <is>
+          <t>Pelvis</t>
+        </is>
+      </c>
+      <c r="G95" s="194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H95" s="195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I95" s="195" t="n"/>
+      <c r="J95" s="178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K95" s="179" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="126" t="n"/>
+      <c r="C96" s="126" t="inlineStr">
         <is>
           <t>Lower Leg</t>
         </is>
       </c>
-      <c r="D94" s="126" t="inlineStr">
+      <c r="D96" s="126" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="E94" s="126" t="inlineStr">
+      <c r="E96" s="126" t="inlineStr">
         <is>
           <t>aPLI</t>
         </is>
       </c>
-      <c r="F94" s="126" t="inlineStr">
+      <c r="F96" s="126" t="inlineStr">
         <is>
           <t>Femur</t>
         </is>
       </c>
-      <c r="G94" s="192" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H94" s="126" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J94" s="156" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K94" s="157" t="n">
+      <c r="G96" s="192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H96" s="126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J96" s="156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K96" s="157" t="n">
         <v>2.5</v>
       </c>
     </row>
-    <row r="95" ht="14.25" customHeight="1" s="129">
-      <c r="A95" s="165" t="n"/>
-      <c r="B95" s="165" t="n"/>
-      <c r="C95" s="165" t="n"/>
-      <c r="D95" s="165" t="n"/>
-      <c r="E95" s="165" t="n"/>
-      <c r="F95" s="165" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="165" t="n"/>
+      <c r="B97" s="165" t="n"/>
+      <c r="C97" s="165" t="n"/>
+      <c r="D97" s="165" t="n"/>
+      <c r="E97" s="165" t="n"/>
+      <c r="F97" s="165" t="inlineStr">
         <is>
           <t>Knee &amp; Tibia</t>
         </is>
       </c>
-      <c r="G95" s="196" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H95" s="197" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I95" s="197" t="n"/>
-      <c r="J95" s="167" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K95" s="168" t="n">
+      <c r="G97" s="196" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H97" s="197" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I97" s="197" t="n"/>
+      <c r="J97" s="167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K97" s="168" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="98" ht="14.25" customHeight="1" s="129">
-      <c r="G98" s="192" t="n"/>
+    <row r="98" ht="14.25" customHeight="1" s="129"/>
+    <row r="100">
+      <c r="G100" s="192" t="n"/>
     </row>
     <row r="1048574" ht="12.75" customHeight="1" s="129"/>
     <row r="1048575" ht="12.75" customHeight="1" s="129"/>
     <row r="1048576" ht="12.75" customHeight="1" s="129"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="S90:S92"/>
-    <mergeCell ref="R90:R92"/>
-    <mergeCell ref="Q90:Q92"/>
+    <mergeCell ref="Q92:Q94"/>
+    <mergeCell ref="S92:S94"/>
+    <mergeCell ref="R92:R94"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>